<commit_message>
various fixes to Estimates, Opportunity, etc. found during production cutover
</commit_message>
<xml_diff>
--- a/uploads/Deal_Tracker_1776401286.xlsx
+++ b/uploads/Deal_Tracker_1776401286.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D9FD00-37D4-471A-A478-456E7C0885AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3298A1-DF3A-4080-9167-200E6F8F5DC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1539,7 +1539,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1611,6 +1611,12 @@
         <fgColor rgb="FFDF2F4A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1624,7 +1630,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1688,6 +1694,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2028,6 +2037,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AY283"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2195,7 +2205,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>48</v>
       </c>
@@ -2351,7 +2361,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>54</v>
       </c>
@@ -2508,7 +2518,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>58</v>
       </c>
@@ -2665,7 +2675,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>60</v>
       </c>
@@ -2819,7 +2829,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>61</v>
       </c>
@@ -2976,7 +2986,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>62</v>
       </c>
@@ -3133,7 +3143,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>64</v>
       </c>
@@ -3290,7 +3300,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>65</v>
       </c>
@@ -3447,7 +3457,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>66</v>
       </c>
@@ -3604,7 +3614,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>71</v>
       </c>
@@ -3760,7 +3770,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>73</v>
       </c>
@@ -3917,7 +3927,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>74</v>
       </c>
@@ -4074,7 +4084,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>75</v>
       </c>
@@ -4231,7 +4241,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>77</v>
       </c>
@@ -4388,7 +4398,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>80</v>
       </c>
@@ -4545,7 +4555,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>82</v>
       </c>
@@ -4702,7 +4712,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>85</v>
       </c>
@@ -4859,7 +4869,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>87</v>
       </c>
@@ -5016,7 +5026,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>89</v>
       </c>
@@ -5173,7 +5183,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>78</v>
       </c>
@@ -5330,7 +5340,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>92</v>
       </c>
@@ -5487,7 +5497,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>93</v>
       </c>
@@ -5643,7 +5653,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>96</v>
       </c>
@@ -5800,7 +5810,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>98</v>
       </c>
@@ -5957,7 +5967,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>99</v>
       </c>
@@ -6114,7 +6124,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="27" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>104</v>
       </c>
@@ -6271,7 +6281,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>105</v>
       </c>
@@ -6428,7 +6438,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>107</v>
       </c>
@@ -6585,7 +6595,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="30" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>108</v>
       </c>
@@ -6742,7 +6752,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>109</v>
       </c>
@@ -6899,7 +6909,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="32" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>112</v>
       </c>
@@ -7056,7 +7066,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>113</v>
       </c>
@@ -7213,7 +7223,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="34" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>115</v>
       </c>
@@ -7370,7 +7380,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="35" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>116</v>
       </c>
@@ -7527,7 +7537,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="36" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>117</v>
       </c>
@@ -7684,7 +7694,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>118</v>
       </c>
@@ -7841,7 +7851,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="38" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>119</v>
       </c>
@@ -7998,7 +8008,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="39" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>120</v>
       </c>
@@ -8155,7 +8165,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="40" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>122</v>
       </c>
@@ -8312,7 +8322,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>124</v>
       </c>
@@ -8469,7 +8479,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="42" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>126</v>
       </c>
@@ -8626,7 +8636,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="43" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>127</v>
       </c>
@@ -8783,7 +8793,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="44" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>128</v>
       </c>
@@ -8940,7 +8950,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>130</v>
       </c>
@@ -9097,7 +9107,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="46" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>134</v>
       </c>
@@ -9254,7 +9264,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>136</v>
       </c>
@@ -9411,7 +9421,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="48" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>138</v>
       </c>
@@ -9568,7 +9578,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="49" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>139</v>
       </c>
@@ -9725,7 +9735,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="50" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>142</v>
       </c>
@@ -9882,7 +9892,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>144</v>
       </c>
@@ -10039,7 +10049,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="52" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>146</v>
       </c>
@@ -10196,7 +10206,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="53" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>148</v>
       </c>
@@ -10353,7 +10363,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="54" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>150</v>
       </c>
@@ -10510,7 +10520,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="55" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>151</v>
       </c>
@@ -10667,7 +10677,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="56" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>153</v>
       </c>
@@ -10824,7 +10834,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="57" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>154</v>
       </c>
@@ -10981,7 +10991,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="58" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>155</v>
       </c>
@@ -11138,7 +11148,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="59" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>156</v>
       </c>
@@ -11295,7 +11305,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="60" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>157</v>
       </c>
@@ -11452,7 +11462,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="61" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>158</v>
       </c>
@@ -11609,7 +11619,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="62" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>159</v>
       </c>
@@ -11766,7 +11776,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="63" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>161</v>
       </c>
@@ -11922,7 +11932,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="64" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>165</v>
       </c>
@@ -12079,7 +12089,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="65" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>166</v>
       </c>
@@ -12236,7 +12246,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="66" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>168</v>
       </c>
@@ -12393,7 +12403,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="67" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>169</v>
       </c>
@@ -12550,7 +12560,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="68" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>170</v>
       </c>
@@ -12706,7 +12716,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="69" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>173</v>
       </c>
@@ -12863,7 +12873,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="70" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>175</v>
       </c>
@@ -13019,7 +13029,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="71" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>178</v>
       </c>
@@ -13176,7 +13186,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="72" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>179</v>
       </c>
@@ -13333,7 +13343,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="73" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>181</v>
       </c>
@@ -13490,7 +13500,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="74" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>183</v>
       </c>
@@ -13646,7 +13656,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="75" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>185</v>
       </c>
@@ -13803,7 +13813,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="76" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>186</v>
       </c>
@@ -13961,7 +13971,7 @@
       </c>
     </row>
     <row r="77" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="2" t="s">
+      <c r="A77" s="22" t="s">
         <v>188</v>
       </c>
       <c r="B77" s="3" t="s">
@@ -14118,7 +14128,7 @@
       </c>
     </row>
     <row r="78" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="2" t="s">
+      <c r="A78" s="22" t="s">
         <v>190</v>
       </c>
       <c r="B78" s="2" t="s">
@@ -15843,7 +15853,7 @@
       </c>
     </row>
     <row r="89" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="2" t="s">
+      <c r="A89" s="22" t="s">
         <v>202</v>
       </c>
       <c r="B89" s="3" t="s">
@@ -15999,7 +16009,7 @@
       </c>
     </row>
     <row r="90" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="2" t="s">
+      <c r="A90" s="22" t="s">
         <v>206</v>
       </c>
       <c r="B90" s="3" t="s">
@@ -16155,7 +16165,7 @@
       </c>
     </row>
     <row r="91" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="2" t="s">
+      <c r="A91" s="22" t="s">
         <v>209</v>
       </c>
       <c r="B91" s="3" t="s">
@@ -16311,7 +16321,7 @@
       </c>
     </row>
     <row r="92" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="2" t="s">
+      <c r="A92" s="22" t="s">
         <v>211</v>
       </c>
       <c r="B92" s="3" t="s">
@@ -16467,7 +16477,7 @@
       </c>
     </row>
     <row r="93" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="2" t="s">
+      <c r="A93" s="22" t="s">
         <v>213</v>
       </c>
       <c r="B93" s="3" t="s">
@@ -16623,7 +16633,7 @@
       </c>
     </row>
     <row r="94" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="2" t="s">
+      <c r="A94" s="22" t="s">
         <v>215</v>
       </c>
       <c r="B94" s="3" t="s">
@@ -16779,7 +16789,7 @@
       </c>
     </row>
     <row r="95" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="2" t="s">
+      <c r="A95" s="22" t="s">
         <v>216</v>
       </c>
       <c r="B95" s="3" t="s">
@@ -16935,7 +16945,7 @@
       </c>
     </row>
     <row r="96" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="2" t="s">
+      <c r="A96" s="22" t="s">
         <v>219</v>
       </c>
       <c r="B96" s="3" t="s">
@@ -17091,7 +17101,7 @@
       </c>
     </row>
     <row r="97" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="2" t="s">
+      <c r="A97" s="22" t="s">
         <v>220</v>
       </c>
       <c r="B97" s="3" t="s">
@@ -17247,7 +17257,7 @@
       </c>
     </row>
     <row r="98" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="2" t="s">
+      <c r="A98" s="22" t="s">
         <v>221</v>
       </c>
       <c r="B98" s="3" t="s">
@@ -17403,7 +17413,7 @@
       </c>
     </row>
     <row r="99" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="2" t="s">
+      <c r="A99" s="22" t="s">
         <v>222</v>
       </c>
       <c r="B99" s="3" t="s">
@@ -17559,7 +17569,7 @@
       </c>
     </row>
     <row r="100" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="2" t="s">
+      <c r="A100" s="22" t="s">
         <v>224</v>
       </c>
       <c r="B100" s="3" t="s">
@@ -17715,7 +17725,7 @@
       </c>
     </row>
     <row r="101" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="2" t="s">
+      <c r="A101" s="22" t="s">
         <v>225</v>
       </c>
       <c r="B101" s="3" t="s">
@@ -17871,7 +17881,7 @@
       </c>
     </row>
     <row r="102" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="2" t="s">
+      <c r="A102" s="22" t="s">
         <v>226</v>
       </c>
       <c r="B102" s="3" t="s">
@@ -18027,7 +18037,7 @@
       </c>
     </row>
     <row r="103" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A103" s="2" t="s">
+      <c r="A103" s="22" t="s">
         <v>228</v>
       </c>
       <c r="B103" s="3" t="s">
@@ -18183,7 +18193,7 @@
       </c>
     </row>
     <row r="104" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A104" s="2" t="s">
+      <c r="A104" s="22" t="s">
         <v>230</v>
       </c>
       <c r="B104" s="3" t="s">
@@ -18339,7 +18349,7 @@
       </c>
     </row>
     <row r="105" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="2" t="s">
+      <c r="A105" s="22" t="s">
         <v>231</v>
       </c>
       <c r="B105" s="3" t="s">
@@ -18495,7 +18505,7 @@
       </c>
     </row>
     <row r="106" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="2" t="s">
+      <c r="A106" s="22" t="s">
         <v>233</v>
       </c>
       <c r="B106" s="3" t="s">
@@ -18651,7 +18661,7 @@
       </c>
     </row>
     <row r="107" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="2" t="s">
+      <c r="A107" s="22" t="s">
         <v>234</v>
       </c>
       <c r="B107" s="3" t="s">
@@ -18807,7 +18817,7 @@
       </c>
     </row>
     <row r="108" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A108" s="2" t="s">
+      <c r="A108" s="22" t="s">
         <v>235</v>
       </c>
       <c r="B108" s="3" t="s">
@@ -18963,7 +18973,7 @@
       </c>
     </row>
     <row r="109" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="2" t="s">
+      <c r="A109" s="22" t="s">
         <v>236</v>
       </c>
       <c r="B109" s="3" t="s">
@@ -19119,7 +19129,7 @@
       </c>
     </row>
     <row r="110" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="2" t="s">
+      <c r="A110" s="22" t="s">
         <v>237</v>
       </c>
       <c r="B110" s="3" t="s">
@@ -19275,7 +19285,7 @@
       </c>
     </row>
     <row r="111" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="2" t="s">
+      <c r="A111" s="22" t="s">
         <v>238</v>
       </c>
       <c r="B111" s="3" t="s">
@@ -19431,7 +19441,7 @@
       </c>
     </row>
     <row r="112" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A112" s="2" t="s">
+      <c r="A112" s="22" t="s">
         <v>241</v>
       </c>
       <c r="B112" s="3" t="s">
@@ -19587,7 +19597,7 @@
       </c>
     </row>
     <row r="113" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="2" t="s">
+      <c r="A113" s="22" t="s">
         <v>242</v>
       </c>
       <c r="B113" s="3" t="s">
@@ -19743,7 +19753,7 @@
       </c>
     </row>
     <row r="114" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="2" t="s">
+      <c r="A114" s="22" t="s">
         <v>244</v>
       </c>
       <c r="B114" s="3" t="s">
@@ -19899,7 +19909,7 @@
       </c>
     </row>
     <row r="115" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="2" t="s">
+      <c r="A115" s="22" t="s">
         <v>246</v>
       </c>
       <c r="B115" s="3" t="s">
@@ -28790,7 +28800,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="172" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
         <v>321</v>
       </c>
@@ -28946,7 +28956,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="173" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
         <v>324</v>
       </c>
@@ -29102,7 +29112,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="174" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
         <v>326</v>
       </c>
@@ -29258,7 +29268,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="175" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
         <v>329</v>
       </c>
@@ -29414,7 +29424,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="176" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
         <v>331</v>
       </c>
@@ -29570,7 +29580,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="177" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
         <v>332</v>
       </c>
@@ -29726,7 +29736,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="178" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="2" t="s">
         <v>333</v>
       </c>
@@ -29882,7 +29892,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="179" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="2" t="s">
         <v>335</v>
       </c>
@@ -30038,7 +30048,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="180" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A180" s="2" t="s">
         <v>338</v>
       </c>
@@ -30194,7 +30204,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="181" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="2" t="s">
         <v>340</v>
       </c>
@@ -30350,7 +30360,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="182" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="2" t="s">
         <v>341</v>
       </c>
@@ -30506,7 +30516,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="183" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A183" s="2" t="s">
         <v>343</v>
       </c>
@@ -30662,7 +30672,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="184" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A184" s="2" t="s">
         <v>345</v>
       </c>
@@ -30818,7 +30828,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="185" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="2" t="s">
         <v>346</v>
       </c>
@@ -30974,7 +30984,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="186" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="2" t="s">
         <v>128</v>
       </c>
@@ -31130,7 +31140,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="187" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A187" s="2" t="s">
         <v>347</v>
       </c>
@@ -31286,7 +31296,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="188" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A188" s="2" t="s">
         <v>349</v>
       </c>
@@ -31442,7 +31452,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="189" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A189" s="2" t="s">
         <v>351</v>
       </c>
@@ -31598,7 +31608,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="190" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="2" t="s">
         <v>352</v>
       </c>
@@ -31754,7 +31764,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="191" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="2" t="s">
         <v>353</v>
       </c>
@@ -31910,7 +31920,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="192" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A192" s="2" t="s">
         <v>355</v>
       </c>
@@ -32066,7 +32076,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="193" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A193" s="2" t="s">
         <v>356</v>
       </c>
@@ -32222,7 +32232,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="194" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="2" t="s">
         <v>357</v>
       </c>
@@ -32378,7 +32388,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="195" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A195" s="2" t="s">
         <v>358</v>
       </c>
@@ -32534,7 +32544,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="196" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A196" s="2" t="s">
         <v>359</v>
       </c>
@@ -32690,7 +32700,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="197" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A197" s="2" t="s">
         <v>360</v>
       </c>
@@ -32846,7 +32856,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="198" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="2" t="s">
         <v>361</v>
       </c>
@@ -33002,7 +33012,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="199" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A199" s="2" t="s">
         <v>362</v>
       </c>
@@ -33158,7 +33168,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="200" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A200" s="2" t="s">
         <v>363</v>
       </c>
@@ -33314,7 +33324,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="201" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A201" s="2" t="s">
         <v>364</v>
       </c>
@@ -33470,7 +33480,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="202" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A202" s="2" t="s">
         <v>365</v>
       </c>
@@ -33626,7 +33636,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="203" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A203" s="2" t="s">
         <v>367</v>
       </c>
@@ -33782,7 +33792,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="204" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A204" s="2" t="s">
         <v>368</v>
       </c>
@@ -33938,7 +33948,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="205" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A205" s="2" t="s">
         <v>369</v>
       </c>
@@ -34094,7 +34104,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="206" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A206" s="2" t="s">
         <v>371</v>
       </c>
@@ -34250,7 +34260,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="207" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A207" s="2" t="s">
         <v>373</v>
       </c>
@@ -34406,7 +34416,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="208" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A208" s="2" t="s">
         <v>374</v>
       </c>
@@ -34562,7 +34572,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="209" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A209" s="2" t="s">
         <v>375</v>
       </c>
@@ -34718,7 +34728,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="210" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A210" s="2" t="s">
         <v>376</v>
       </c>
@@ -34874,7 +34884,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="211" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A211" s="2" t="s">
         <v>377</v>
       </c>
@@ -35030,7 +35040,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="212" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A212" s="2" t="s">
         <v>378</v>
       </c>
@@ -35186,7 +35196,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="213" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A213" s="2" t="s">
         <v>379</v>
       </c>
@@ -35342,7 +35352,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="214" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A214" s="2" t="s">
         <v>380</v>
       </c>
@@ -35498,7 +35508,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="215" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A215" s="2" t="s">
         <v>381</v>
       </c>
@@ -35654,7 +35664,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="216" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A216" s="2" t="s">
         <v>382</v>
       </c>
@@ -35810,7 +35820,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="217" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A217" s="2" t="s">
         <v>383</v>
       </c>
@@ -35966,7 +35976,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="218" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A218" s="2" t="s">
         <v>384</v>
       </c>
@@ -36122,7 +36132,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="219" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A219" s="2" t="s">
         <v>385</v>
       </c>
@@ -36278,7 +36288,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="220" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A220" s="2" t="s">
         <v>386</v>
       </c>
@@ -36434,7 +36444,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="221" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A221" s="2" t="s">
         <v>387</v>
       </c>
@@ -36590,7 +36600,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="222" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A222" s="2" t="s">
         <v>388</v>
       </c>
@@ -36746,7 +36756,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="223" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A223" s="2" t="s">
         <v>390</v>
       </c>
@@ -36902,7 +36912,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="224" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A224" s="2" t="s">
         <v>392</v>
       </c>
@@ -37058,7 +37068,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="225" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A225" s="2" t="s">
         <v>394</v>
       </c>
@@ -37214,7 +37224,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="226" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A226" s="2" t="s">
         <v>395</v>
       </c>
@@ -37370,7 +37380,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="227" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A227" s="2" t="s">
         <v>396</v>
       </c>
@@ -37526,7 +37536,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="228" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A228" s="2" t="s">
         <v>397</v>
       </c>
@@ -37682,7 +37692,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="229" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A229" s="2" t="s">
         <v>398</v>
       </c>
@@ -37838,7 +37848,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="230" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A230" s="2" t="s">
         <v>399</v>
       </c>
@@ -37994,7 +38004,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="231" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A231" s="2" t="s">
         <v>401</v>
       </c>
@@ -38150,7 +38160,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="232" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A232" s="2" t="s">
         <v>403</v>
       </c>
@@ -38306,7 +38316,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="233" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A233" s="2" t="s">
         <v>404</v>
       </c>
@@ -38462,7 +38472,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="234" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A234" s="2" t="s">
         <v>143</v>
       </c>
@@ -38618,7 +38628,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="235" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A235" s="2" t="s">
         <v>405</v>
       </c>
@@ -38774,7 +38784,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="236" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A236" s="2" t="s">
         <v>407</v>
       </c>
@@ -38930,7 +38940,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="237" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A237" s="2" t="s">
         <v>409</v>
       </c>
@@ -39086,7 +39096,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="238" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A238" s="2" t="s">
         <v>410</v>
       </c>
@@ -39242,7 +39252,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="239" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A239" s="2" t="s">
         <v>412</v>
       </c>
@@ -39398,7 +39408,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="240" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A240" s="2" t="s">
         <v>414</v>
       </c>
@@ -39554,7 +39564,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="241" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A241" s="2" t="s">
         <v>415</v>
       </c>
@@ -39710,7 +39720,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="242" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A242" s="2" t="s">
         <v>417</v>
       </c>
@@ -39866,7 +39876,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="243" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A243" s="2" t="s">
         <v>418</v>
       </c>
@@ -40022,7 +40032,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="244" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A244" s="2" t="s">
         <v>419</v>
       </c>
@@ -40178,7 +40188,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="245" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A245" s="2" t="s">
         <v>421</v>
       </c>
@@ -40334,7 +40344,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="246" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A246" s="2" t="s">
         <v>422</v>
       </c>
@@ -40490,7 +40500,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="247" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A247" s="2" t="s">
         <v>114</v>
       </c>
@@ -40646,7 +40656,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="248" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A248" s="2" t="s">
         <v>424</v>
       </c>
@@ -40802,7 +40812,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="249" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A249" s="2" t="s">
         <v>425</v>
       </c>
@@ -40958,7 +40968,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="250" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A250" s="2" t="s">
         <v>426</v>
       </c>
@@ -41114,7 +41124,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="251" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A251" s="2" t="s">
         <v>427</v>
       </c>
@@ -41270,7 +41280,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="252" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A252" s="2" t="s">
         <v>428</v>
       </c>
@@ -41426,7 +41436,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="253" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A253" s="2" t="s">
         <v>429</v>
       </c>
@@ -41582,7 +41592,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="254" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A254" s="2" t="s">
         <v>430</v>
       </c>
@@ -41738,7 +41748,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="255" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A255" s="2" t="s">
         <v>431</v>
       </c>
@@ -41894,7 +41904,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="256" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A256" s="2" t="s">
         <v>432</v>
       </c>
@@ -42050,7 +42060,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="257" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A257" s="2" t="s">
         <v>434</v>
       </c>
@@ -42206,7 +42216,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="258" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A258" s="2" t="s">
         <v>435</v>
       </c>
@@ -42362,7 +42372,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="259" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A259" s="2" t="s">
         <v>436</v>
       </c>
@@ -42518,7 +42528,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="260" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A260" s="2" t="s">
         <v>437</v>
       </c>
@@ -42674,7 +42684,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="261" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A261" s="2" t="s">
         <v>439</v>
       </c>
@@ -42830,7 +42840,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="262" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A262" s="2" t="s">
         <v>441</v>
       </c>
@@ -42986,7 +42996,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="263" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A263" s="2" t="s">
         <v>442</v>
       </c>
@@ -43142,7 +43152,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="264" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A264" s="2" t="s">
         <v>443</v>
       </c>
@@ -43298,7 +43308,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="265" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A265" s="2" t="s">
         <v>445</v>
       </c>
@@ -43454,7 +43464,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="266" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A266" s="2" t="s">
         <v>447</v>
       </c>
@@ -43610,7 +43620,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="267" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A267" s="2" t="s">
         <v>449</v>
       </c>
@@ -43766,7 +43776,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="268" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A268" s="2" t="s">
         <v>145</v>
       </c>
@@ -43922,7 +43932,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="269" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A269" s="2" t="s">
         <v>450</v>
       </c>
@@ -44078,7 +44088,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="270" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A270" s="2" t="s">
         <v>452</v>
       </c>
@@ -44234,7 +44244,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="271" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A271" s="2" t="s">
         <v>454</v>
       </c>
@@ -44390,7 +44400,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="272" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A272" s="2" t="s">
         <v>455</v>
       </c>
@@ -44546,7 +44556,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="273" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A273" s="2" t="s">
         <v>456</v>
       </c>
@@ -44702,7 +44712,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="274" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A274" s="2" t="s">
         <v>457</v>
       </c>
@@ -44858,7 +44868,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="275" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A275" s="2" t="s">
         <v>459</v>
       </c>
@@ -45014,7 +45024,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="276" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A276" s="2" t="s">
         <v>461</v>
       </c>
@@ -45170,7 +45180,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="277" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A277" s="2" t="s">
         <v>463</v>
       </c>
@@ -45326,7 +45336,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="278" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A278" s="2" t="s">
         <v>464</v>
       </c>
@@ -45482,7 +45492,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="279" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A279" s="2" t="s">
         <v>465</v>
       </c>
@@ -45638,7 +45648,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="280" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A280" s="2" t="s">
         <v>466</v>
       </c>
@@ -45794,7 +45804,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="281" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A281" s="2" t="s">
         <v>468</v>
       </c>
@@ -45950,7 +45960,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="282" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:51" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A282" s="2" t="s">
         <v>469</v>
       </c>
@@ -46108,7 +46118,15 @@
     </row>
     <row r="283" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A1:AY282" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AY282" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Negotiation"/>
+        <filter val="Proposal"/>
+        <filter val="Won"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>

</xml_diff>

<commit_message>
various fixes from production cutover
</commit_message>
<xml_diff>
--- a/uploads/Deal_Tracker_1776401286.xlsx
+++ b/uploads/Deal_Tracker_1776401286.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3298A1-DF3A-4080-9167-200E6F8F5DC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E72342C9-5EC8-4F0F-AF35-884072C9A19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="deal tracker" sheetId="1" r:id="rId1"/>
@@ -20065,7 +20065,7 @@
       </c>
     </row>
     <row r="116" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="2" t="s">
+      <c r="A116" s="22" t="s">
         <v>249</v>
       </c>
       <c r="B116" s="3" t="s">
@@ -20221,7 +20221,7 @@
       </c>
     </row>
     <row r="117" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="2" t="s">
+      <c r="A117" s="22" t="s">
         <v>251</v>
       </c>
       <c r="B117" s="3" t="s">
@@ -20377,7 +20377,7 @@
       </c>
     </row>
     <row r="118" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="2" t="s">
+      <c r="A118" s="22" t="s">
         <v>252</v>
       </c>
       <c r="B118" s="3" t="s">
@@ -20533,7 +20533,7 @@
       </c>
     </row>
     <row r="119" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A119" s="2" t="s">
+      <c r="A119" s="22" t="s">
         <v>253</v>
       </c>
       <c r="B119" s="3" t="s">
@@ -20689,7 +20689,7 @@
       </c>
     </row>
     <row r="120" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="2" t="s">
+      <c r="A120" s="22" t="s">
         <v>254</v>
       </c>
       <c r="B120" s="3" t="s">
@@ -20845,7 +20845,7 @@
       </c>
     </row>
     <row r="121" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A121" s="2" t="s">
+      <c r="A121" s="22" t="s">
         <v>255</v>
       </c>
       <c r="B121" s="3" t="s">
@@ -21001,7 +21001,7 @@
       </c>
     </row>
     <row r="122" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="2" t="s">
+      <c r="A122" s="22" t="s">
         <v>256</v>
       </c>
       <c r="B122" s="3" t="s">
@@ -21157,7 +21157,7 @@
       </c>
     </row>
     <row r="123" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="2" t="s">
+      <c r="A123" s="22" t="s">
         <v>257</v>
       </c>
       <c r="B123" s="3" t="s">
@@ -21313,7 +21313,7 @@
       </c>
     </row>
     <row r="124" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="2" t="s">
+      <c r="A124" s="22" t="s">
         <v>258</v>
       </c>
       <c r="B124" s="3" t="s">
@@ -21469,7 +21469,7 @@
       </c>
     </row>
     <row r="125" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="2" t="s">
+      <c r="A125" s="22" t="s">
         <v>259</v>
       </c>
       <c r="B125" s="3" t="s">
@@ -21625,7 +21625,7 @@
       </c>
     </row>
     <row r="126" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="2" t="s">
+      <c r="A126" s="22" t="s">
         <v>260</v>
       </c>
       <c r="B126" s="3" t="s">
@@ -21781,7 +21781,7 @@
       </c>
     </row>
     <row r="127" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A127" s="2" t="s">
+      <c r="A127" s="22" t="s">
         <v>262</v>
       </c>
       <c r="B127" s="3" t="s">
@@ -21937,7 +21937,7 @@
       </c>
     </row>
     <row r="128" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="2" t="s">
+      <c r="A128" s="22" t="s">
         <v>264</v>
       </c>
       <c r="B128" s="3" t="s">
@@ -22093,7 +22093,7 @@
       </c>
     </row>
     <row r="129" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="2" t="s">
+      <c r="A129" s="22" t="s">
         <v>265</v>
       </c>
       <c r="B129" s="3" t="s">
@@ -22249,7 +22249,7 @@
       </c>
     </row>
     <row r="130" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="2" t="s">
+      <c r="A130" s="22" t="s">
         <v>266</v>
       </c>
       <c r="B130" s="3" t="s">
@@ -22405,7 +22405,7 @@
       </c>
     </row>
     <row r="131" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A131" s="2" t="s">
+      <c r="A131" s="22" t="s">
         <v>267</v>
       </c>
       <c r="B131" s="3" t="s">
@@ -22561,7 +22561,7 @@
       </c>
     </row>
     <row r="132" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A132" s="2" t="s">
+      <c r="A132" s="22" t="s">
         <v>268</v>
       </c>
       <c r="B132" s="3" t="s">
@@ -22717,7 +22717,7 @@
       </c>
     </row>
     <row r="133" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A133" s="2" t="s">
+      <c r="A133" s="22" t="s">
         <v>269</v>
       </c>
       <c r="B133" s="3" t="s">
@@ -22873,7 +22873,7 @@
       </c>
     </row>
     <row r="134" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A134" s="2" t="s">
+      <c r="A134" s="22" t="s">
         <v>270</v>
       </c>
       <c r="B134" s="3" t="s">
@@ -23029,7 +23029,7 @@
       </c>
     </row>
     <row r="135" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="2" t="s">
+      <c r="A135" s="22" t="s">
         <v>272</v>
       </c>
       <c r="B135" s="3" t="s">
@@ -23185,7 +23185,7 @@
       </c>
     </row>
     <row r="136" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="2" t="s">
+      <c r="A136" s="22" t="s">
         <v>273</v>
       </c>
       <c r="B136" s="3" t="s">
@@ -23341,7 +23341,7 @@
       </c>
     </row>
     <row r="137" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="2" t="s">
+      <c r="A137" s="22" t="s">
         <v>274</v>
       </c>
       <c r="B137" s="3" t="s">
@@ -23497,7 +23497,7 @@
       </c>
     </row>
     <row r="138" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="2" t="s">
+      <c r="A138" s="22" t="s">
         <v>275</v>
       </c>
       <c r="B138" s="3" t="s">
@@ -23653,7 +23653,7 @@
       </c>
     </row>
     <row r="139" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A139" s="2" t="s">
+      <c r="A139" s="22" t="s">
         <v>277</v>
       </c>
       <c r="B139" s="3" t="s">
@@ -23809,7 +23809,7 @@
       </c>
     </row>
     <row r="140" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="2" t="s">
+      <c r="A140" s="22" t="s">
         <v>278</v>
       </c>
       <c r="B140" s="3" t="s">
@@ -23965,7 +23965,7 @@
       </c>
     </row>
     <row r="141" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A141" s="2" t="s">
+      <c r="A141" s="22" t="s">
         <v>280</v>
       </c>
       <c r="B141" s="3" t="s">
@@ -24121,7 +24121,7 @@
       </c>
     </row>
     <row r="142" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A142" s="2" t="s">
+      <c r="A142" s="22" t="s">
         <v>282</v>
       </c>
       <c r="B142" s="3" t="s">
@@ -24277,7 +24277,7 @@
       </c>
     </row>
     <row r="143" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A143" s="2" t="s">
+      <c r="A143" s="22" t="s">
         <v>283</v>
       </c>
       <c r="B143" s="3" t="s">
@@ -24433,7 +24433,7 @@
       </c>
     </row>
     <row r="144" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A144" s="2" t="s">
+      <c r="A144" s="22" t="s">
         <v>284</v>
       </c>
       <c r="B144" s="3" t="s">
@@ -24589,7 +24589,7 @@
       </c>
     </row>
     <row r="145" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A145" s="2" t="s">
+      <c r="A145" s="22" t="s">
         <v>285</v>
       </c>
       <c r="B145" s="3" t="s">
@@ -24745,7 +24745,7 @@
       </c>
     </row>
     <row r="146" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A146" s="2" t="s">
+      <c r="A146" s="22" t="s">
         <v>287</v>
       </c>
       <c r="B146" s="3" t="s">
@@ -24901,7 +24901,7 @@
       </c>
     </row>
     <row r="147" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="2" t="s">
+      <c r="A147" s="22" t="s">
         <v>288</v>
       </c>
       <c r="B147" s="3" t="s">
@@ -25057,7 +25057,7 @@
       </c>
     </row>
     <row r="148" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A148" s="2" t="s">
+      <c r="A148" s="22" t="s">
         <v>289</v>
       </c>
       <c r="B148" s="3" t="s">
@@ -25213,7 +25213,7 @@
       </c>
     </row>
     <row r="149" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="2" t="s">
+      <c r="A149" s="22" t="s">
         <v>290</v>
       </c>
       <c r="B149" s="3" t="s">
@@ -25369,7 +25369,7 @@
       </c>
     </row>
     <row r="150" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="2" t="s">
+      <c r="A150" s="22" t="s">
         <v>292</v>
       </c>
       <c r="B150" s="3" t="s">
@@ -25525,7 +25525,7 @@
       </c>
     </row>
     <row r="151" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A151" s="2" t="s">
+      <c r="A151" s="22" t="s">
         <v>293</v>
       </c>
       <c r="B151" s="3" t="s">
@@ -25681,7 +25681,7 @@
       </c>
     </row>
     <row r="152" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A152" s="2" t="s">
+      <c r="A152" s="22" t="s">
         <v>294</v>
       </c>
       <c r="B152" s="3" t="s">
@@ -25837,7 +25837,7 @@
       </c>
     </row>
     <row r="153" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A153" s="2" t="s">
+      <c r="A153" s="22" t="s">
         <v>296</v>
       </c>
       <c r="B153" s="3" t="s">
@@ -25993,7 +25993,7 @@
       </c>
     </row>
     <row r="154" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="2" t="s">
+      <c r="A154" s="22" t="s">
         <v>298</v>
       </c>
       <c r="B154" s="3" t="s">
@@ -26149,7 +26149,7 @@
       </c>
     </row>
     <row r="155" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A155" s="2" t="s">
+      <c r="A155" s="22" t="s">
         <v>300</v>
       </c>
       <c r="B155" s="3" t="s">
@@ -26305,7 +26305,7 @@
       </c>
     </row>
     <row r="156" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A156" s="2" t="s">
+      <c r="A156" s="22" t="s">
         <v>301</v>
       </c>
       <c r="B156" s="3" t="s">
@@ -26461,7 +26461,7 @@
       </c>
     </row>
     <row r="157" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A157" s="2" t="s">
+      <c r="A157" s="22" t="s">
         <v>303</v>
       </c>
       <c r="B157" s="3" t="s">
@@ -26617,7 +26617,7 @@
       </c>
     </row>
     <row r="158" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A158" s="2" t="s">
+      <c r="A158" s="22" t="s">
         <v>305</v>
       </c>
       <c r="B158" s="3" t="s">
@@ -26773,7 +26773,7 @@
       </c>
     </row>
     <row r="159" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A159" s="2" t="s">
+      <c r="A159" s="22" t="s">
         <v>306</v>
       </c>
       <c r="B159" s="3" t="s">
@@ -26929,7 +26929,7 @@
       </c>
     </row>
     <row r="160" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A160" s="2" t="s">
+      <c r="A160" s="22" t="s">
         <v>307</v>
       </c>
       <c r="B160" s="3" t="s">
@@ -27085,7 +27085,7 @@
       </c>
     </row>
     <row r="161" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A161" s="2" t="s">
+      <c r="A161" s="22" t="s">
         <v>308</v>
       </c>
       <c r="B161" s="3" t="s">
@@ -27241,7 +27241,7 @@
       </c>
     </row>
     <row r="162" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A162" s="2" t="s">
+      <c r="A162" s="22" t="s">
         <v>309</v>
       </c>
       <c r="B162" s="3" t="s">
@@ -27397,7 +27397,7 @@
       </c>
     </row>
     <row r="163" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A163" s="2" t="s">
+      <c r="A163" s="22" t="s">
         <v>310</v>
       </c>
       <c r="B163" s="3" t="s">
@@ -27553,7 +27553,7 @@
       </c>
     </row>
     <row r="164" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A164" s="2" t="s">
+      <c r="A164" s="22" t="s">
         <v>311</v>
       </c>
       <c r="B164" s="3" t="s">
@@ -27709,7 +27709,7 @@
       </c>
     </row>
     <row r="165" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A165" s="2" t="s">
+      <c r="A165" s="22" t="s">
         <v>312</v>
       </c>
       <c r="B165" s="3" t="s">
@@ -27865,7 +27865,7 @@
       </c>
     </row>
     <row r="166" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A166" s="2" t="s">
+      <c r="A166" s="22" t="s">
         <v>313</v>
       </c>
       <c r="B166" s="3" t="s">
@@ -28021,7 +28021,7 @@
       </c>
     </row>
     <row r="167" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A167" s="2" t="s">
+      <c r="A167" s="22" t="s">
         <v>314</v>
       </c>
       <c r="B167" s="3" t="s">
@@ -28177,7 +28177,7 @@
       </c>
     </row>
     <row r="168" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A168" s="2" t="s">
+      <c r="A168" s="22" t="s">
         <v>315</v>
       </c>
       <c r="B168" s="3" t="s">
@@ -28333,7 +28333,7 @@
       </c>
     </row>
     <row r="169" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A169" s="2" t="s">
+      <c r="A169" s="22" t="s">
         <v>317</v>
       </c>
       <c r="B169" s="3" t="s">
@@ -28489,7 +28489,7 @@
       </c>
     </row>
     <row r="170" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A170" s="2" t="s">
+      <c r="A170" s="22" t="s">
         <v>318</v>
       </c>
       <c r="B170" s="3" t="s">
@@ -28645,7 +28645,7 @@
       </c>
     </row>
     <row r="171" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A171" s="2" t="s">
+      <c r="A171" s="22" t="s">
         <v>319</v>
       </c>
       <c r="B171" s="3" t="s">

</xml_diff>

<commit_message>
large set of corrections as part of cutover defects
</commit_message>
<xml_diff>
--- a/uploads/Deal_Tracker_1776401286.xlsx
+++ b/uploads/Deal_Tracker_1776401286.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E72342C9-5EC8-4F0F-AF35-884072C9A19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{69A7B597-4ABB-4EFB-BAE5-4D9E6838A117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="deal tracker" sheetId="1" r:id="rId1"/>
@@ -14,6 +14,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'deal tracker'!$A$1:$AY$282</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -11967,7 +11968,7 @@
         <v>49</v>
       </c>
       <c r="L64" s="19">
-        <f t="shared" ref="L64:L67" si="4">EDATE(I64,3)</f>
+        <f>EDATE(I64,3)</f>
         <v>46218</v>
       </c>
       <c r="M64" s="6">
@@ -12124,7 +12125,7 @@
         <v>49</v>
       </c>
       <c r="L65" s="19">
-        <f t="shared" si="4"/>
+        <f>EDATE(I65,3)</f>
         <v>46218</v>
       </c>
       <c r="M65" s="6">
@@ -12281,7 +12282,7 @@
         <v>49</v>
       </c>
       <c r="L66" s="19">
-        <f t="shared" si="4"/>
+        <f>EDATE(I66,3)</f>
         <v>46002</v>
       </c>
       <c r="M66" s="6">
@@ -12438,11 +12439,11 @@
         <v>49</v>
       </c>
       <c r="L67" s="19">
-        <f t="shared" si="4"/>
+        <f>EDATE(I67,3)</f>
         <v>45797</v>
       </c>
       <c r="M67" s="6">
-        <f t="shared" ref="M67:M130" si="5">EDATE(L67,INT(P67)) + (P67-INT(P67)) * DAY(EOMONTH(EDATE(L67,INT(P67)),0))</f>
+        <f t="shared" ref="M67:M130" si="4">EDATE(L67,INT(P67)) + (P67-INT(P67)) * DAY(EOMONTH(EDATE(L67,INT(P67)),0))</f>
         <v>45812.5</v>
       </c>
       <c r="N67" t="s">
@@ -12598,7 +12599,7 @@
         <v>46023</v>
       </c>
       <c r="M68" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46038.5</v>
       </c>
       <c r="N68" s="3" t="s">
@@ -12755,7 +12756,7 @@
         <v>46131</v>
       </c>
       <c r="M69" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46146</v>
       </c>
       <c r="N69" t="s">
@@ -12911,7 +12912,7 @@
         <v>46143</v>
       </c>
       <c r="M70" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46508</v>
       </c>
       <c r="N70" s="3" t="s">
@@ -13064,11 +13065,11 @@
         <v>49</v>
       </c>
       <c r="L71" s="19">
-        <f t="shared" ref="L71:L73" si="6">EDATE(I71,3)</f>
+        <f>EDATE(I71,3)</f>
         <v>46192</v>
       </c>
       <c r="M71" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46207</v>
       </c>
       <c r="N71" t="s">
@@ -13221,11 +13222,11 @@
         <v>49</v>
       </c>
       <c r="L72" s="19">
-        <f t="shared" si="6"/>
+        <f>EDATE(I72,3)</f>
         <v>46203</v>
       </c>
       <c r="M72" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46218</v>
       </c>
       <c r="N72" t="s">
@@ -13378,11 +13379,11 @@
         <v>49</v>
       </c>
       <c r="L73" s="19">
-        <f t="shared" si="6"/>
+        <f>EDATE(I73,3)</f>
         <v>46203</v>
       </c>
       <c r="M73" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46218</v>
       </c>
       <c r="N73" t="s">
@@ -13538,7 +13539,7 @@
         <v>46113</v>
       </c>
       <c r="M74" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46478</v>
       </c>
       <c r="N74" s="3" t="s">
@@ -13691,11 +13692,11 @@
         <v>49</v>
       </c>
       <c r="L75" s="19">
-        <f t="shared" ref="L75:L86" si="7">EDATE(I75,3)</f>
+        <f t="shared" ref="L75:L86" si="5">EDATE(I75,3)</f>
         <v>46132</v>
       </c>
       <c r="M75" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46147</v>
       </c>
       <c r="N75" t="s">
@@ -13848,11 +13849,11 @@
         <v>49</v>
       </c>
       <c r="L76" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>46164</v>
       </c>
       <c r="M76" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46179.5</v>
       </c>
       <c r="N76" t="s">
@@ -13971,7 +13972,7 @@
       </c>
     </row>
     <row r="77" spans="1:51" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="22" t="s">
+      <c r="A77" s="2" t="s">
         <v>188</v>
       </c>
       <c r="B77" s="3" t="s">
@@ -14005,11 +14006,11 @@
         <v>49</v>
       </c>
       <c r="L77" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>46203</v>
       </c>
       <c r="M77" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46218</v>
       </c>
       <c r="N77" t="s">
@@ -14162,11 +14163,11 @@
         <v>49</v>
       </c>
       <c r="L78" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>46186</v>
       </c>
       <c r="M78" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46201</v>
       </c>
       <c r="N78" t="s">
@@ -14319,11 +14320,11 @@
         <v>49</v>
       </c>
       <c r="L79" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>46070</v>
       </c>
       <c r="M79" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46084</v>
       </c>
       <c r="N79" t="s">
@@ -14476,11 +14477,11 @@
         <v>49</v>
       </c>
       <c r="L80" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>46111</v>
       </c>
       <c r="M80" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46126.5</v>
       </c>
       <c r="N80" t="s">
@@ -14633,11 +14634,11 @@
         <v>49</v>
       </c>
       <c r="L81" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>46111</v>
       </c>
       <c r="M81" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46126.5</v>
       </c>
       <c r="N81" t="s">
@@ -14790,11 +14791,11 @@
         <v>46038</v>
       </c>
       <c r="L82" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>46052</v>
       </c>
       <c r="M82" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46067.5</v>
       </c>
       <c r="N82" t="s">
@@ -14947,11 +14948,11 @@
         <v>46038</v>
       </c>
       <c r="L83" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>46052</v>
       </c>
       <c r="M83" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46067.5</v>
       </c>
       <c r="N83" t="s">
@@ -15104,11 +15105,11 @@
         <v>46038</v>
       </c>
       <c r="L84" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>46070</v>
       </c>
       <c r="M84" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46084</v>
       </c>
       <c r="N84" t="s">
@@ -15261,11 +15262,11 @@
         <v>46038</v>
       </c>
       <c r="L85" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>46070</v>
       </c>
       <c r="M85" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46084</v>
       </c>
       <c r="N85" t="s">
@@ -15418,11 +15419,11 @@
         <v>46038</v>
       </c>
       <c r="L86" s="19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>46052</v>
       </c>
       <c r="M86" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46067.5</v>
       </c>
       <c r="N86" t="s">
@@ -15578,7 +15579,7 @@
         <v>46143</v>
       </c>
       <c r="M87" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46508</v>
       </c>
       <c r="N87" s="3" t="s">
@@ -15734,7 +15735,7 @@
         <v>46143</v>
       </c>
       <c r="M88" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46327</v>
       </c>
       <c r="N88" s="3" t="s">
@@ -15890,7 +15891,7 @@
         <v>46082</v>
       </c>
       <c r="M89" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>46097.5</v>
       </c>
       <c r="N89" s="3" t="s">
@@ -16046,7 +16047,7 @@
         <v>45139</v>
       </c>
       <c r="M90" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45154.5</v>
       </c>
       <c r="N90" t="s">
@@ -16202,7 +16203,7 @@
         <v>45139</v>
       </c>
       <c r="M91" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45154.5</v>
       </c>
       <c r="N91" t="s">
@@ -16358,7 +16359,7 @@
         <v>45231</v>
       </c>
       <c r="M92" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45246</v>
       </c>
       <c r="N92" t="s">
@@ -16514,7 +16515,7 @@
         <v>45332</v>
       </c>
       <c r="M93" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45346.5</v>
       </c>
       <c r="N93" t="s">
@@ -16670,7 +16671,7 @@
         <v>45323</v>
       </c>
       <c r="M94" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45337.5</v>
       </c>
       <c r="N94" t="s">
@@ -16826,7 +16827,7 @@
         <v>45352</v>
       </c>
       <c r="M95" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45367.5</v>
       </c>
       <c r="N95" t="s">
@@ -16982,7 +16983,7 @@
         <v>45352</v>
       </c>
       <c r="M96" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45367.5</v>
       </c>
       <c r="N96" t="s">
@@ -17138,7 +17139,7 @@
         <v>45352</v>
       </c>
       <c r="M97" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45367.5</v>
       </c>
       <c r="N97" t="s">
@@ -17294,7 +17295,7 @@
         <v>45383</v>
       </c>
       <c r="M98" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45398</v>
       </c>
       <c r="N98" t="s">
@@ -17450,7 +17451,7 @@
         <v>45413</v>
       </c>
       <c r="M99" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45428.5</v>
       </c>
       <c r="N99" t="s">
@@ -17606,7 +17607,7 @@
         <v>45444</v>
       </c>
       <c r="M100" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45459</v>
       </c>
       <c r="N100" t="s">
@@ -17762,7 +17763,7 @@
         <v>45444</v>
       </c>
       <c r="M101" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45459</v>
       </c>
       <c r="N101" t="s">
@@ -17918,7 +17919,7 @@
         <v>45474</v>
       </c>
       <c r="M102" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45489.5</v>
       </c>
       <c r="N102" t="s">
@@ -18074,7 +18075,7 @@
         <v>45474</v>
       </c>
       <c r="M103" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45489.5</v>
       </c>
       <c r="N103" s="3" t="s">
@@ -18230,7 +18231,7 @@
         <v>45505</v>
       </c>
       <c r="M104" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45520.5</v>
       </c>
       <c r="N104" t="s">
@@ -18386,7 +18387,7 @@
         <v>45536</v>
       </c>
       <c r="M105" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45551</v>
       </c>
       <c r="N105" t="s">
@@ -18542,7 +18543,7 @@
         <v>45597</v>
       </c>
       <c r="M106" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45612</v>
       </c>
       <c r="N106" t="s">
@@ -18698,7 +18699,7 @@
         <v>45597</v>
       </c>
       <c r="M107" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45612</v>
       </c>
       <c r="N107" t="s">
@@ -18854,7 +18855,7 @@
         <v>45627</v>
       </c>
       <c r="M108" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45642.5</v>
       </c>
       <c r="N108" t="s">
@@ -19010,7 +19011,7 @@
         <v>45627</v>
       </c>
       <c r="M109" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45642.5</v>
       </c>
       <c r="N109" t="s">
@@ -19166,7 +19167,7 @@
         <v>45627</v>
       </c>
       <c r="M110" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45642.5</v>
       </c>
       <c r="N110" t="s">
@@ -19322,7 +19323,7 @@
         <v>45717</v>
       </c>
       <c r="M111" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45732.5</v>
       </c>
       <c r="N111" t="s">
@@ -19478,7 +19479,7 @@
         <v>45748</v>
       </c>
       <c r="M112" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45763</v>
       </c>
       <c r="N112" s="3" t="s">
@@ -19634,7 +19635,7 @@
         <v>45170</v>
       </c>
       <c r="M113" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45185</v>
       </c>
       <c r="N113" t="s">
@@ -19790,7 +19791,7 @@
         <v>45323</v>
       </c>
       <c r="M114" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45337.5</v>
       </c>
       <c r="N114" t="s">
@@ -19946,7 +19947,7 @@
         <v>45261</v>
       </c>
       <c r="M115" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45276.5</v>
       </c>
       <c r="N115" t="s">
@@ -20102,7 +20103,7 @@
         <v>45352</v>
       </c>
       <c r="M116" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45367.5</v>
       </c>
       <c r="N116" t="s">
@@ -20258,7 +20259,7 @@
         <v>45444</v>
       </c>
       <c r="M117" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45459</v>
       </c>
       <c r="N117" t="s">
@@ -20414,7 +20415,7 @@
         <v>45413</v>
       </c>
       <c r="M118" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45428.5</v>
       </c>
       <c r="N118" t="s">
@@ -20570,7 +20571,7 @@
         <v>45474</v>
       </c>
       <c r="M119" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45489.5</v>
       </c>
       <c r="N119" t="s">
@@ -20726,7 +20727,7 @@
         <v>45536</v>
       </c>
       <c r="M120" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45551</v>
       </c>
       <c r="N120" t="s">
@@ -20882,7 +20883,7 @@
         <v>45536</v>
       </c>
       <c r="M121" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45551</v>
       </c>
       <c r="N121" t="s">
@@ -21038,7 +21039,7 @@
         <v>45597</v>
       </c>
       <c r="M122" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45612</v>
       </c>
       <c r="N122" t="s">
@@ -21194,7 +21195,7 @@
         <v>45597</v>
       </c>
       <c r="M123" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45612</v>
       </c>
       <c r="N123" t="s">
@@ -21350,7 +21351,7 @@
         <v>45597</v>
       </c>
       <c r="M124" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45612</v>
       </c>
       <c r="N124" t="s">
@@ -21506,7 +21507,7 @@
         <v>45597</v>
       </c>
       <c r="M125" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45612</v>
       </c>
       <c r="N125" t="s">
@@ -21662,7 +21663,7 @@
         <v>45717</v>
       </c>
       <c r="M126" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45732.5</v>
       </c>
       <c r="N126" t="s">
@@ -21818,7 +21819,7 @@
         <v>45717</v>
       </c>
       <c r="M127" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45732.5</v>
       </c>
       <c r="N127" s="3" t="s">
@@ -21974,7 +21975,7 @@
         <v>45748</v>
       </c>
       <c r="M128" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45763</v>
       </c>
       <c r="N128" t="s">
@@ -22130,7 +22131,7 @@
         <v>45778</v>
       </c>
       <c r="M129" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45793.5</v>
       </c>
       <c r="N129" t="s">
@@ -22286,7 +22287,7 @@
         <v>45778</v>
       </c>
       <c r="M130" s="6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>45793.5</v>
       </c>
       <c r="N130" t="s">
@@ -22442,7 +22443,7 @@
         <v>45778</v>
       </c>
       <c r="M131" s="6">
-        <f t="shared" ref="M131:M194" si="8">EDATE(L131,INT(P131)) + (P131-INT(P131)) * DAY(EOMONTH(EDATE(L131,INT(P131)),0))</f>
+        <f t="shared" ref="M131:M194" si="6">EDATE(L131,INT(P131)) + (P131-INT(P131)) * DAY(EOMONTH(EDATE(L131,INT(P131)),0))</f>
         <v>45793.5</v>
       </c>
       <c r="N131" t="s">
@@ -22598,7 +22599,7 @@
         <v>45809</v>
       </c>
       <c r="M132" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45824</v>
       </c>
       <c r="N132" s="3" t="s">
@@ -22754,7 +22755,7 @@
         <v>45809</v>
       </c>
       <c r="M133" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45824</v>
       </c>
       <c r="N133" t="s">
@@ -22910,7 +22911,7 @@
         <v>45839</v>
       </c>
       <c r="M134" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46447</v>
       </c>
       <c r="N134" s="3" t="s">
@@ -23066,7 +23067,7 @@
         <v>45839</v>
       </c>
       <c r="M135" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45854.5</v>
       </c>
       <c r="N135" s="3" t="s">
@@ -23222,7 +23223,7 @@
         <v>45839</v>
       </c>
       <c r="M136" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45854.5</v>
       </c>
       <c r="N136" t="s">
@@ -23378,7 +23379,7 @@
         <v>45870</v>
       </c>
       <c r="M137" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45885.5</v>
       </c>
       <c r="N137" t="s">
@@ -23534,7 +23535,7 @@
         <v>45870</v>
       </c>
       <c r="M138" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45885.5</v>
       </c>
       <c r="N138" s="3" t="s">
@@ -23690,7 +23691,7 @@
         <v>45870</v>
       </c>
       <c r="M139" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45885.5</v>
       </c>
       <c r="N139" s="3" t="s">
@@ -23846,7 +23847,7 @@
         <v>45870</v>
       </c>
       <c r="M140" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45885.5</v>
       </c>
       <c r="N140" s="3" t="s">
@@ -24002,7 +24003,7 @@
         <v>45901</v>
       </c>
       <c r="M141" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45916</v>
       </c>
       <c r="N141" s="3" t="s">
@@ -24158,7 +24159,7 @@
         <v>45901</v>
       </c>
       <c r="M142" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45916</v>
       </c>
       <c r="N142" s="3" t="s">
@@ -24314,7 +24315,7 @@
         <v>45931</v>
       </c>
       <c r="M143" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45946.5</v>
       </c>
       <c r="N143" t="s">
@@ -24470,7 +24471,7 @@
         <v>45931</v>
       </c>
       <c r="M144" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45946.5</v>
       </c>
       <c r="N144" t="s">
@@ -24626,7 +24627,7 @@
         <v>45962</v>
       </c>
       <c r="M145" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45977</v>
       </c>
       <c r="N145" s="3" t="s">
@@ -24782,7 +24783,7 @@
         <v>45931</v>
       </c>
       <c r="M146" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45946.5</v>
       </c>
       <c r="N146" t="s">
@@ -24938,7 +24939,7 @@
         <v>45931</v>
       </c>
       <c r="M147" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45946.5</v>
       </c>
       <c r="N147" t="s">
@@ -25094,7 +25095,7 @@
         <v>45962</v>
       </c>
       <c r="M148" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45977</v>
       </c>
       <c r="N148" s="3" t="s">
@@ -25250,7 +25251,7 @@
         <v>45992</v>
       </c>
       <c r="M149" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46007.5</v>
       </c>
       <c r="N149" s="3" t="s">
@@ -25406,7 +25407,7 @@
         <v>45992</v>
       </c>
       <c r="M150" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46007.5</v>
       </c>
       <c r="N150" s="3" t="s">
@@ -25562,7 +25563,7 @@
         <v>45962</v>
       </c>
       <c r="M151" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46327</v>
       </c>
       <c r="N151" s="3" t="s">
@@ -25718,7 +25719,7 @@
         <v>45962</v>
       </c>
       <c r="M152" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45977</v>
       </c>
       <c r="N152" s="3" t="s">
@@ -25874,7 +25875,7 @@
         <v>45992</v>
       </c>
       <c r="M153" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46023</v>
       </c>
       <c r="N153" s="3" t="s">
@@ -26030,7 +26031,7 @@
         <v>46054</v>
       </c>
       <c r="M154" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46419</v>
       </c>
       <c r="N154" s="3" t="s">
@@ -26186,7 +26187,7 @@
         <v>46023</v>
       </c>
       <c r="M155" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46113</v>
       </c>
       <c r="N155" s="3" t="s">
@@ -26342,7 +26343,7 @@
         <v>46023</v>
       </c>
       <c r="M156" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46082</v>
       </c>
       <c r="N156" s="3" t="s">
@@ -26498,7 +26499,7 @@
         <v>46082</v>
       </c>
       <c r="M157" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46266</v>
       </c>
       <c r="N157" s="3" t="s">
@@ -26654,7 +26655,7 @@
         <v>46023</v>
       </c>
       <c r="M158" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46388</v>
       </c>
       <c r="N158" s="3" t="s">
@@ -26810,7 +26811,7 @@
         <v>46023</v>
       </c>
       <c r="M159" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46174</v>
       </c>
       <c r="N159" s="3" t="s">
@@ -26966,7 +26967,7 @@
         <v>46023</v>
       </c>
       <c r="M160" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46038.5</v>
       </c>
       <c r="N160" t="s">
@@ -27122,7 +27123,7 @@
         <v>46023</v>
       </c>
       <c r="M161" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46174</v>
       </c>
       <c r="N161" s="3" t="s">
@@ -27278,7 +27279,7 @@
         <v>46082</v>
       </c>
       <c r="M162" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46113</v>
       </c>
       <c r="N162" s="3" t="s">
@@ -27434,7 +27435,7 @@
         <v>46082</v>
       </c>
       <c r="M163" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46174</v>
       </c>
       <c r="N163" s="3" t="s">
@@ -27590,7 +27591,7 @@
         <v>46113</v>
       </c>
       <c r="M164" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46174</v>
       </c>
       <c r="N164" s="3" t="s">
@@ -27746,7 +27747,7 @@
         <v>46113</v>
       </c>
       <c r="M165" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46204</v>
       </c>
       <c r="N165" s="3" t="s">
@@ -27902,7 +27903,7 @@
         <v>46082</v>
       </c>
       <c r="M166" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46174</v>
       </c>
       <c r="N166" s="3" t="s">
@@ -28058,7 +28059,7 @@
         <v>46113</v>
       </c>
       <c r="M167" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46478</v>
       </c>
       <c r="N167" s="3" t="s">
@@ -28214,7 +28215,7 @@
         <v>46113</v>
       </c>
       <c r="M168" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46174</v>
       </c>
       <c r="N168" s="3" t="s">
@@ -28370,7 +28371,7 @@
         <v>46113</v>
       </c>
       <c r="M169" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46204</v>
       </c>
       <c r="N169" s="3" t="s">
@@ -28526,7 +28527,7 @@
         <v>46143</v>
       </c>
       <c r="M170" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46419</v>
       </c>
       <c r="N170" s="3" t="s">
@@ -28682,7 +28683,7 @@
         <v>46113</v>
       </c>
       <c r="M171" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46478</v>
       </c>
       <c r="N171" s="3" t="s">
@@ -28838,7 +28839,7 @@
         <v>45078</v>
       </c>
       <c r="M172" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45093</v>
       </c>
       <c r="N172" t="s">
@@ -28994,7 +28995,7 @@
         <v>45200</v>
       </c>
       <c r="M173" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45215.5</v>
       </c>
       <c r="N173" t="s">
@@ -29150,7 +29151,7 @@
         <v>45323</v>
       </c>
       <c r="M174" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45337.5</v>
       </c>
       <c r="N174" t="s">
@@ -29306,7 +29307,7 @@
         <v>45352</v>
       </c>
       <c r="M175" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45367.5</v>
       </c>
       <c r="N175" t="s">
@@ -29462,7 +29463,7 @@
         <v>45352</v>
       </c>
       <c r="M176" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45367.5</v>
       </c>
       <c r="N176" t="s">
@@ -29618,7 +29619,7 @@
         <v>45717</v>
       </c>
       <c r="M177" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45732.5</v>
       </c>
       <c r="N177" t="s">
@@ -29774,7 +29775,7 @@
         <v>45717</v>
       </c>
       <c r="M178" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45732.5</v>
       </c>
       <c r="N178" t="s">
@@ -29930,7 +29931,7 @@
         <v>45566</v>
       </c>
       <c r="M179" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45581.5</v>
       </c>
       <c r="N179" t="s">
@@ -30086,7 +30087,7 @@
         <v>45597</v>
       </c>
       <c r="M180" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45612</v>
       </c>
       <c r="N180" t="s">
@@ -30242,7 +30243,7 @@
         <v>45597</v>
       </c>
       <c r="M181" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45612</v>
       </c>
       <c r="N181" t="s">
@@ -30398,7 +30399,7 @@
         <v>45597</v>
       </c>
       <c r="M182" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45612</v>
       </c>
       <c r="N182" t="s">
@@ -30554,7 +30555,7 @@
         <v>45597</v>
       </c>
       <c r="M183" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45612</v>
       </c>
       <c r="N183" t="s">
@@ -30710,7 +30711,7 @@
         <v>45717</v>
       </c>
       <c r="M184" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45732.5</v>
       </c>
       <c r="N184" t="s">
@@ -30866,7 +30867,7 @@
         <v>45658</v>
       </c>
       <c r="M185" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45673.5</v>
       </c>
       <c r="N185" t="s">
@@ -31022,7 +31023,7 @@
         <v>45658</v>
       </c>
       <c r="M186" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45673.5</v>
       </c>
       <c r="N186" t="s">
@@ -31178,7 +31179,7 @@
         <v>45717</v>
       </c>
       <c r="M187" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45732.5</v>
       </c>
       <c r="N187" t="s">
@@ -31334,7 +31335,7 @@
         <v>45717</v>
       </c>
       <c r="M188" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45732.5</v>
       </c>
       <c r="N188" t="s">
@@ -31490,7 +31491,7 @@
         <v>45717</v>
       </c>
       <c r="M189" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45732.5</v>
       </c>
       <c r="N189" t="s">
@@ -31646,7 +31647,7 @@
         <v>45717</v>
       </c>
       <c r="M190" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45732.5</v>
       </c>
       <c r="N190" t="s">
@@ -31802,7 +31803,7 @@
         <v>45717</v>
       </c>
       <c r="M191" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45732.5</v>
       </c>
       <c r="N191" t="s">
@@ -31958,7 +31959,7 @@
         <v>45717</v>
       </c>
       <c r="M192" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45732.5</v>
       </c>
       <c r="N192" t="s">
@@ -32114,7 +32115,7 @@
         <v>45748</v>
       </c>
       <c r="M193" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45763</v>
       </c>
       <c r="N193" t="s">
@@ -32270,7 +32271,7 @@
         <v>45748</v>
       </c>
       <c r="M194" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45763</v>
       </c>
       <c r="N194" t="s">
@@ -32426,7 +32427,7 @@
         <v>45748</v>
       </c>
       <c r="M195" s="6">
-        <f t="shared" ref="M195:M258" si="9">EDATE(L195,INT(P195)) + (P195-INT(P195)) * DAY(EOMONTH(EDATE(L195,INT(P195)),0))</f>
+        <f t="shared" ref="M195:M258" si="7">EDATE(L195,INT(P195)) + (P195-INT(P195)) * DAY(EOMONTH(EDATE(L195,INT(P195)),0))</f>
         <v>45763</v>
       </c>
       <c r="N195" t="s">
@@ -32582,7 +32583,7 @@
         <v>45778</v>
       </c>
       <c r="M196" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N196" t="s">
@@ -32738,7 +32739,7 @@
         <v>45778</v>
       </c>
       <c r="M197" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N197" t="s">
@@ -32894,7 +32895,7 @@
         <v>45778</v>
       </c>
       <c r="M198" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N198" t="s">
@@ -33050,7 +33051,7 @@
         <v>45778</v>
       </c>
       <c r="M199" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N199" t="s">
@@ -33206,7 +33207,7 @@
         <v>45778</v>
       </c>
       <c r="M200" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N200" t="s">
@@ -33362,7 +33363,7 @@
         <v>45778</v>
       </c>
       <c r="M201" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N201" t="s">
@@ -33518,7 +33519,7 @@
         <v>45352</v>
       </c>
       <c r="M202" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45367.5</v>
       </c>
       <c r="N202" t="s">
@@ -33674,7 +33675,7 @@
         <v>45444</v>
       </c>
       <c r="M203" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45459</v>
       </c>
       <c r="N203" t="s">
@@ -33830,7 +33831,7 @@
         <v>45444</v>
       </c>
       <c r="M204" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45459</v>
       </c>
       <c r="N204" t="s">
@@ -33986,7 +33987,7 @@
         <v>45778</v>
       </c>
       <c r="M205" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N205" t="s">
@@ -34142,7 +34143,7 @@
         <v>45444</v>
       </c>
       <c r="M206" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45459</v>
       </c>
       <c r="N206" t="s">
@@ -34298,7 +34299,7 @@
         <v>45778</v>
       </c>
       <c r="M207" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N207" t="s">
@@ -34454,7 +34455,7 @@
         <v>45505</v>
       </c>
       <c r="M208" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45520.5</v>
       </c>
       <c r="N208" t="s">
@@ -34610,7 +34611,7 @@
         <v>45778</v>
       </c>
       <c r="M209" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N209" t="s">
@@ -34766,7 +34767,7 @@
         <v>45505</v>
       </c>
       <c r="M210" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45520.5</v>
       </c>
       <c r="N210" t="s">
@@ -34922,7 +34923,7 @@
         <v>45536</v>
       </c>
       <c r="M211" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45551</v>
       </c>
       <c r="N211" t="s">
@@ -35078,7 +35079,7 @@
         <v>45536</v>
       </c>
       <c r="M212" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45551</v>
       </c>
       <c r="N212" t="s">
@@ -35234,7 +35235,7 @@
         <v>45778</v>
       </c>
       <c r="M213" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N213" t="s">
@@ -35390,7 +35391,7 @@
         <v>45566</v>
       </c>
       <c r="M214" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45581.5</v>
       </c>
       <c r="N214" t="s">
@@ -35546,7 +35547,7 @@
         <v>45566</v>
       </c>
       <c r="M215" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45581.5</v>
       </c>
       <c r="N215" t="s">
@@ -35702,7 +35703,7 @@
         <v>45778</v>
       </c>
       <c r="M216" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N216" t="s">
@@ -35858,7 +35859,7 @@
         <v>45778</v>
       </c>
       <c r="M217" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N217" t="s">
@@ -36014,7 +36015,7 @@
         <v>45778</v>
       </c>
       <c r="M218" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N218" t="s">
@@ -36170,7 +36171,7 @@
         <v>45778</v>
       </c>
       <c r="M219" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N219" t="s">
@@ -36326,7 +36327,7 @@
         <v>45778</v>
       </c>
       <c r="M220" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N220" t="s">
@@ -36482,7 +36483,7 @@
         <v>45323</v>
       </c>
       <c r="M221" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45337.5</v>
       </c>
       <c r="N221" t="s">
@@ -36638,7 +36639,7 @@
         <v>45323</v>
       </c>
       <c r="M222" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45337.5</v>
       </c>
       <c r="N222" t="s">
@@ -36794,7 +36795,7 @@
         <v>45323</v>
       </c>
       <c r="M223" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45337.5</v>
       </c>
       <c r="N223" t="s">
@@ -36950,7 +36951,7 @@
         <v>45323</v>
       </c>
       <c r="M224" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45337.5</v>
       </c>
       <c r="N224" t="s">
@@ -37106,7 +37107,7 @@
         <v>45778</v>
       </c>
       <c r="M225" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N225" t="s">
@@ -37262,7 +37263,7 @@
         <v>45597</v>
       </c>
       <c r="M226" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45612</v>
       </c>
       <c r="N226" t="s">
@@ -37418,7 +37419,7 @@
         <v>45597</v>
       </c>
       <c r="M227" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45612</v>
       </c>
       <c r="N227" t="s">
@@ -37574,7 +37575,7 @@
         <v>45778</v>
       </c>
       <c r="M228" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N228" t="s">
@@ -37730,7 +37731,7 @@
         <v>45627</v>
       </c>
       <c r="M229" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45642.5</v>
       </c>
       <c r="N229" t="s">
@@ -37886,7 +37887,7 @@
         <v>45627</v>
       </c>
       <c r="M230" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45642.5</v>
       </c>
       <c r="N230" t="s">
@@ -38042,7 +38043,7 @@
         <v>45689</v>
       </c>
       <c r="M231" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45703</v>
       </c>
       <c r="N231" t="s">
@@ -38198,7 +38199,7 @@
         <v>45689</v>
       </c>
       <c r="M232" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45703</v>
       </c>
       <c r="N232" t="s">
@@ -38354,7 +38355,7 @@
         <v>45778</v>
       </c>
       <c r="M233" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N233" t="s">
@@ -38510,7 +38511,7 @@
         <v>45778</v>
       </c>
       <c r="M234" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N234" t="s">
@@ -38666,7 +38667,7 @@
         <v>45778</v>
       </c>
       <c r="M235" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N235" t="s">
@@ -38822,7 +38823,7 @@
         <v>45778</v>
       </c>
       <c r="M236" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N236" t="s">
@@ -38978,7 +38979,7 @@
         <v>45778</v>
       </c>
       <c r="M237" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N237" t="s">
@@ -39134,7 +39135,7 @@
         <v>45778</v>
       </c>
       <c r="M238" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N238" t="s">
@@ -39290,7 +39291,7 @@
         <v>45778</v>
       </c>
       <c r="M239" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N239" t="s">
@@ -39446,7 +39447,7 @@
         <v>45778</v>
       </c>
       <c r="M240" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N240" t="s">
@@ -39602,7 +39603,7 @@
         <v>45778</v>
       </c>
       <c r="M241" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N241" t="s">
@@ -39758,7 +39759,7 @@
         <v>45778</v>
       </c>
       <c r="M242" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N242" t="s">
@@ -39914,7 +39915,7 @@
         <v>45778</v>
       </c>
       <c r="M243" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N243" t="s">
@@ -40070,7 +40071,7 @@
         <v>45778</v>
       </c>
       <c r="M244" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N244" t="s">
@@ -40226,7 +40227,7 @@
         <v>45778</v>
       </c>
       <c r="M245" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N245" t="s">
@@ -40382,7 +40383,7 @@
         <v>45778</v>
       </c>
       <c r="M246" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N246" t="s">
@@ -40538,7 +40539,7 @@
         <v>45778</v>
       </c>
       <c r="M247" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45793.5</v>
       </c>
       <c r="N247" t="s">
@@ -40694,7 +40695,7 @@
         <v>45809</v>
       </c>
       <c r="M248" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45824</v>
       </c>
       <c r="N248" t="s">
@@ -40850,7 +40851,7 @@
         <v>45839</v>
       </c>
       <c r="M249" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45854.5</v>
       </c>
       <c r="N249" t="s">
@@ -41006,7 +41007,7 @@
         <v>45870</v>
       </c>
       <c r="M250" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45885.5</v>
       </c>
       <c r="N250" t="s">
@@ -41162,7 +41163,7 @@
         <v>45870</v>
       </c>
       <c r="M251" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45885.5</v>
       </c>
       <c r="N251" t="s">
@@ -41318,7 +41319,7 @@
         <v>45870</v>
       </c>
       <c r="M252" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45885.5</v>
       </c>
       <c r="N252" t="s">
@@ -41474,7 +41475,7 @@
         <v>45901</v>
       </c>
       <c r="M253" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45916</v>
       </c>
       <c r="N253" t="s">
@@ -41630,7 +41631,7 @@
         <v>45931</v>
       </c>
       <c r="M254" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45946.5</v>
       </c>
       <c r="N254" t="s">
@@ -41786,7 +41787,7 @@
         <v>45931</v>
       </c>
       <c r="M255" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45946.5</v>
       </c>
       <c r="N255" t="s">
@@ -41942,7 +41943,7 @@
         <v>45931</v>
       </c>
       <c r="M256" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45946.5</v>
       </c>
       <c r="N256" t="s">
@@ -42098,7 +42099,7 @@
         <v>45962</v>
       </c>
       <c r="M257" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45977</v>
       </c>
       <c r="N257" s="3" t="s">
@@ -42254,7 +42255,7 @@
         <v>45962</v>
       </c>
       <c r="M258" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>45977</v>
       </c>
       <c r="N258" t="s">
@@ -42410,7 +42411,7 @@
         <v>45962</v>
       </c>
       <c r="M259" s="6">
-        <f t="shared" ref="M259:M282" si="10">EDATE(L259,INT(P259)) + (P259-INT(P259)) * DAY(EOMONTH(EDATE(L259,INT(P259)),0))</f>
+        <f t="shared" ref="M259:M282" si="8">EDATE(L259,INT(P259)) + (P259-INT(P259)) * DAY(EOMONTH(EDATE(L259,INT(P259)),0))</f>
         <v>45977</v>
       </c>
       <c r="N259" t="s">
@@ -42566,7 +42567,7 @@
         <v>45962</v>
       </c>
       <c r="M260" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>45977</v>
       </c>
       <c r="N260" t="s">
@@ -42722,7 +42723,7 @@
         <v>45931</v>
       </c>
       <c r="M261" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>45946.5</v>
       </c>
       <c r="N261" s="3" t="s">
@@ -42878,7 +42879,7 @@
         <v>46054</v>
       </c>
       <c r="M262" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46068</v>
       </c>
       <c r="N262" t="s">
@@ -43034,7 +43035,7 @@
         <v>46054</v>
       </c>
       <c r="M263" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46068</v>
       </c>
       <c r="N263" t="s">
@@ -43190,7 +43191,7 @@
         <v>46054</v>
       </c>
       <c r="M264" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46082</v>
       </c>
       <c r="N264" s="3" t="s">
@@ -43346,7 +43347,7 @@
         <v>46082</v>
       </c>
       <c r="M265" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46097.5</v>
       </c>
       <c r="N265" t="s">
@@ -43502,7 +43503,7 @@
         <v>46082</v>
       </c>
       <c r="M266" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46097.5</v>
       </c>
       <c r="N266" t="s">
@@ -43658,7 +43659,7 @@
         <v>46082</v>
       </c>
       <c r="M267" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46097.5</v>
       </c>
       <c r="N267" t="s">
@@ -43814,7 +43815,7 @@
         <v>46082</v>
       </c>
       <c r="M268" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46097.5</v>
       </c>
       <c r="N268" t="s">
@@ -43970,7 +43971,7 @@
         <v>46082</v>
       </c>
       <c r="M269" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46097.5</v>
       </c>
       <c r="N269" t="s">
@@ -44126,7 +44127,7 @@
         <v>46082</v>
       </c>
       <c r="M270" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46097.5</v>
       </c>
       <c r="N270" t="s">
@@ -44282,7 +44283,7 @@
         <v>46082</v>
       </c>
       <c r="M271" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46097.5</v>
       </c>
       <c r="N271" t="s">
@@ -44438,7 +44439,7 @@
         <v>46082</v>
       </c>
       <c r="M272" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46097.5</v>
       </c>
       <c r="N272" t="s">
@@ -44594,7 +44595,7 @@
         <v>46082</v>
       </c>
       <c r="M273" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46097.5</v>
       </c>
       <c r="N273" t="s">
@@ -44750,7 +44751,7 @@
         <v>46082</v>
       </c>
       <c r="M274" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46097.5</v>
       </c>
       <c r="N274" t="s">
@@ -44906,7 +44907,7 @@
         <v>46113</v>
       </c>
       <c r="M275" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46128</v>
       </c>
       <c r="N275" t="s">
@@ -45062,7 +45063,7 @@
         <v>46113</v>
       </c>
       <c r="M276" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46128</v>
       </c>
       <c r="N276" s="3" t="s">
@@ -45218,7 +45219,7 @@
         <v>46113</v>
       </c>
       <c r="M277" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46128</v>
       </c>
       <c r="N277" t="s">
@@ -45374,7 +45375,7 @@
         <v>46113</v>
       </c>
       <c r="M278" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46128</v>
       </c>
       <c r="N278" t="s">
@@ -45530,7 +45531,7 @@
         <v>46113</v>
       </c>
       <c r="M279" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46128</v>
       </c>
       <c r="N279" t="s">
@@ -45686,7 +45687,7 @@
         <v>46113</v>
       </c>
       <c r="M280" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>46128</v>
       </c>
       <c r="N280" t="s">
@@ -45842,7 +45843,7 @@
         <v>45931</v>
       </c>
       <c r="M281" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>45946.5</v>
       </c>
       <c r="N281" s="3" t="s">
@@ -45998,7 +45999,7 @@
         <v>45931</v>
       </c>
       <c r="M282" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>45946.5</v>
       </c>
       <c r="N282" t="s">

</xml_diff>